<commit_message>
code and db updated also db backups
</commit_message>
<xml_diff>
--- a/10aug2026/Surveyv + Gpx.xlsx
+++ b/10aug2026/Surveyv + Gpx.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Barqaab\10aug2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E77642C0-4D62-410A-ACC9-C0806D88CD71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{787F8AD2-9B2F-4F0A-8031-2D34DEBF32DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HtSurveyForm - 081025" sheetId="1" r:id="rId1"/>
@@ -113,7 +113,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3427" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3445" uniqueCount="264">
   <si>
     <t>Data Form for HT (GIS Survey Barqaab - PPL - OMS Consortium)</t>
   </si>
@@ -907,6 +907,60 @@
   <si>
     <t>ag_con</t>
   </si>
+  <si>
+    <t>2/0 AWG</t>
+  </si>
+  <si>
+    <t>4/0 AWG</t>
+  </si>
+  <si>
+    <t>500 MCM</t>
+  </si>
+  <si>
+    <t>ANT</t>
+  </si>
+  <si>
+    <t>DOG</t>
+  </si>
+  <si>
+    <t>GOPHER</t>
+  </si>
+  <si>
+    <t>OSPREY</t>
+  </si>
+  <si>
+    <t>PANTHER</t>
+  </si>
+  <si>
+    <t>RABBIT</t>
+  </si>
+  <si>
+    <t>WASP</t>
+  </si>
+  <si>
+    <t>220 MM</t>
+  </si>
+  <si>
+    <t>240 MM</t>
+  </si>
+  <si>
+    <t>120 MCM</t>
+  </si>
+  <si>
+    <t>350 MCM</t>
+  </si>
+  <si>
+    <t>240 MCM</t>
+  </si>
+  <si>
+    <t>Steel Wire</t>
+  </si>
+  <si>
+    <t>T Wire</t>
+  </si>
+  <si>
+    <t>Telephone Pole</t>
+  </si>
 </sst>
 </file>
 
@@ -1261,7 +1315,7 @@
     <xf numFmtId="0" fontId="13" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1519,6 +1573,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Accent2" xfId="4" builtinId="33"/>
@@ -2030,7 +2086,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
-      <xdr:colOff>508000</xdr:colOff>
+      <xdr:colOff>49389</xdr:colOff>
       <xdr:row>46</xdr:row>
       <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
@@ -2112,15 +2168,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>44450</xdr:rowOff>
+      <xdr:colOff>311150</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>143228</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>77</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
+      <xdr:colOff>330200</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>39158</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2143,8 +2199,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8591550" y="9436100"/>
-          <a:ext cx="1238250" cy="4867275"/>
+          <a:off x="8806039" y="9682339"/>
+          <a:ext cx="1232605" cy="4848930"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3953,8 +4009,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB10EE2-F4C9-4D62-AA1D-041CAE80A87C}">
-  <dimension ref="F28:P51"/>
+  <dimension ref="F28:S71"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="19" max="19" width="15.26953125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="28" spans="6:8">
       <c r="F28" t="s">
@@ -3982,7 +4041,7 @@
       <c r="O43" s="99"/>
       <c r="P43" s="99"/>
     </row>
-    <row r="50" spans="12:16" ht="14.5" customHeight="1">
+    <row r="50" spans="12:19" ht="14.5" customHeight="1">
       <c r="L50" s="100" t="s">
         <v>184</v>
       </c>
@@ -3993,12 +4052,102 @@
       </c>
       <c r="P50" s="99"/>
     </row>
-    <row r="51" spans="12:16">
+    <row r="51" spans="12:19">
       <c r="L51" s="100"/>
       <c r="M51" s="100"/>
       <c r="N51" s="100"/>
       <c r="O51" s="99"/>
       <c r="P51" s="99"/>
+    </row>
+    <row r="54" spans="12:19">
+      <c r="S54" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="55" spans="12:19">
+      <c r="S55" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="56" spans="12:19">
+      <c r="S56" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="57" spans="12:19">
+      <c r="S57" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="58" spans="12:19">
+      <c r="S58" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="59" spans="12:19">
+      <c r="S59" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="60" spans="12:19">
+      <c r="S60" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="61" spans="12:19">
+      <c r="S61" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="62" spans="12:19">
+      <c r="S62" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="63" spans="12:19">
+      <c r="S63" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="64" spans="12:19">
+      <c r="S64" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="65" spans="19:19">
+      <c r="S65" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="66" spans="19:19">
+      <c r="S66" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="67" spans="19:19">
+      <c r="S67" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="68" spans="19:19">
+      <c r="S68" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="69" spans="19:19">
+      <c r="S69" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="70" spans="19:19">
+      <c r="S70" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="71" spans="19:19">
+      <c r="S71" t="s">
+        <v>263</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4128,7 +4277,7 @@
       </c>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="104"/>
+      <c r="A27" s="113"/>
       <c r="B27" s="104"/>
       <c r="C27" s="104"/>
       <c r="D27" s="104"/>
@@ -4136,10 +4285,10 @@
       <c r="F27" s="104"/>
     </row>
     <row r="37" spans="1:6">
-      <c r="A37" s="103" t="s">
+      <c r="A37" s="114"/>
+      <c r="B37" s="103" t="s">
         <v>192</v>
       </c>
-      <c r="B37" s="103"/>
       <c r="C37" s="103"/>
       <c r="D37" s="103"/>
       <c r="E37" s="103"/>
@@ -4362,9 +4511,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B19:F19"/>
-    <mergeCell ref="A37:F37"/>
     <mergeCell ref="A45:F45"/>
     <mergeCell ref="A55:F55"/>
+    <mergeCell ref="B37:F37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>